<commit_message>
agentic-qe-mvp: Flow 2 = Epic 8 AQPI-32 + Epic 6 AQPI-23 revised for release 2.0 (AQPI-24/25 changed, new AQPI-37); release-2.0 Jira export snapshot
Co-Authored-By: Devin AI <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/agentic-qe-mvp/demo-artifacts/comparison/compare-CYC-1-vs-CYC-4.xlsx
+++ b/agentic-qe-mvp/demo-artifacts/comparison/compare-CYC-1-vs-CYC-4.xlsx
@@ -43,7 +43,7 @@
     <t>Requirements</t>
   </si>
   <si>
-    <t>REQ-129, REQ-130, REQ-131, REQ-132</t>
+    <t>REQ-129, REQ-130, REQ-131, REQ-132, REQ-133, REQ-134, REQ-135, REQ-136, REQ-137, REQ-138</t>
   </si>
   <si>
     <t>REQ-122, REQ-124, REQ-126</t>
@@ -52,7 +52,7 @@
     <t>Test cases</t>
   </si>
   <si>
-    <t>TC-F-129, TC-F-130, TC-F-131, TC-F-132, TC-F-133</t>
+    <t>TC-F-129, TC-F-130, TC-F-131, TC-F-132, TC-F-133, TC-F-134, TC-F-135, TC-F-136, TC-F-137, TC-F-138, TC-F-139, TC-F-140</t>
   </si>
   <si>
     <t>TC-F-112, TC-F-115, TC-F-119, TC-F-120, TC-F-121, TC-F-122</t>
@@ -61,7 +61,7 @@
     <t>Scripts</t>
   </si>
   <si>
-    <t>br-131-free-cancellation.spec.js, br-132-cancellation-outcome.spec.js</t>
+    <t>br-131-free-cancellation.spec.js, br-132-cancellation-outcome.spec.js, br-133-non-refundable-cancellation.spec.js, br-134-cancellation-deadline-email.spec.js, br-135-ops-retry-limit.spec.js, br-136-cancellation-email.spec.js, br-137-cancellation-email-failure.spec.js</t>
   </si>
   <si>
     <t>br-122-cart-expiry.spec.js, br-124-resend-limit.spec.js, br-126-stay-length-limit.spec.js</t>
@@ -576,10 +576,10 @@
         <v>128</v>
       </c>
       <c r="C2" s="2">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="D2" s="2">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="E2" s="2">
         <v>3</v>
@@ -602,10 +602,10 @@
         <v>132</v>
       </c>
       <c r="C3" s="2">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="D3" s="2">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="E3" s="2">
         <v>6</v>
@@ -628,10 +628,10 @@
         <v>58</v>
       </c>
       <c r="C4" s="2">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="D4" s="2">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E4" s="2">
         <v>3</v>
@@ -739,7 +739,7 @@
         <v>74</v>
       </c>
       <c r="C2" s="2">
-        <v>77</v>
+        <v>83</v>
       </c>
     </row>
     <row r="3" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -750,7 +750,7 @@
         <v>74</v>
       </c>
       <c r="C3" s="2">
-        <v>76</v>
+        <v>82</v>
       </c>
     </row>
     <row r="4" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -772,7 +772,7 @@
         <v>100</v>
       </c>
       <c r="C5" s="2">
-        <v>98.7</v>
+        <v>98.8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Defect lifecycle: release 1.0 has 3 real defects (AQPI-4, AQPI-17, AQPI-21); release 2.0 fixes AQPI-4, which Flow 2 retests and certifies closed, and adds 2 new defects (AQPI-34, AQPI-25); @rule [AQPI-n] tags link code rules to their story
Co-Authored-By: Devin AI <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/agentic-qe-mvp/demo-artifacts/comparison/compare-CYC-1-vs-CYC-4.xlsx
+++ b/agentic-qe-mvp/demo-artifacts/comparison/compare-CYC-1-vs-CYC-4.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="46">
   <si>
     <t>Artifact</t>
   </si>
@@ -127,22 +127,31 @@
     <t>CYC-1 defects</t>
   </si>
   <si>
-    <t/>
+    <t>DEF-001, DEF-002, DEF-003</t>
   </si>
   <si>
     <t>CYC-4 defects</t>
   </si>
   <si>
-    <t>DEF-001</t>
+    <t>DEF-001, DEF-002, DEF-007, DEF-008</t>
   </si>
   <si>
     <t>new</t>
   </si>
   <si>
+    <t>DEF-007, DEF-008</t>
+  </si>
+  <si>
     <t>still open</t>
   </si>
   <si>
+    <t>DEF-001, DEF-002</t>
+  </si>
+  <si>
     <t>resolved</t>
+  </si>
+  <si>
+    <t>DEF-003</t>
   </si>
 </sst>
 </file>
@@ -747,10 +756,10 @@
         <v>31</v>
       </c>
       <c r="B3" s="2">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="C3" s="2">
-        <v>82</v>
+        <v>79</v>
       </c>
     </row>
     <row r="4" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -758,10 +767,10 @@
         <v>32</v>
       </c>
       <c r="B4" s="2">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C4" s="2">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -769,10 +778,10 @@
         <v>33</v>
       </c>
       <c r="B5" s="2">
-        <v>100</v>
+        <v>95.9</v>
       </c>
       <c r="C5" s="2">
-        <v>98.8</v>
+        <v>95.2</v>
       </c>
     </row>
   </sheetData>
@@ -819,23 +828,23 @@
         <v>40</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
     </row>
     <row r="6" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>